<commit_message>
revised manuscript, added legends to main figures
</commit_message>
<xml_diff>
--- a/tables/Table1_Species_protemics_Summary_table_rev7.xlsx
+++ b/tables/Table1_Species_protemics_Summary_table_rev7.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/211a55de1c355a5b/Projects/BucklerLab/Tripsacum_freezing_tolerance/manuscript_V2/1_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/211a55de1c355a5b/Projects/BucklerLab/PACMAD-Rhizome-Proteomics/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{3D108CAD-EFD0-5441-84A0-8060CACB3BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F74B8655-8EE0-EA43-ABB8-2384B0E0B8FF}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{3D108CAD-EFD0-5441-84A0-8060CACB3BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F976B7E-DC08-7F4A-8012-5E78D3B36AE7}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="38280" windowHeight="24580" activeTab="1" xr2:uid="{E31260A5-6BF7-4247-931C-1F444D52B9F8}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" activeTab="1" xr2:uid="{E31260A5-6BF7-4247-931C-1F444D52B9F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
   <si>
     <t>Species</t>
   </si>
@@ -265,6 +265,19 @@
     </r>
   </si>
   <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Proteins quantified</t>
+  </si>
+  <si>
+    <t>Shared Winter/Summer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,468
+</t>
+  </si>
+  <si>
     <r>
       <t>T. dactyloides '</t>
     </r>
@@ -272,7 +285,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>KS'</t>
@@ -282,7 +295,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> × T. floridanium</t>
@@ -294,7 +307,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">T. dactyloides </t>
@@ -303,7 +316,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>'IA'</t>
@@ -313,7 +326,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
@@ -322,7 +335,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>×</t>
@@ -332,7 +345,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> T. dactyloides</t>
@@ -341,7 +354,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 'FL'</t>
@@ -353,7 +366,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. dactyloides</t>
@@ -362,7 +375,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 'MO' × </t>
@@ -372,7 +385,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. dactyloides</t>
@@ -381,7 +394,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 'TX'</t>
@@ -393,7 +406,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. dactyloides</t>
@@ -402,7 +415,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 'IL' × </t>
@@ -412,7 +425,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. floridanium</t>
@@ -424,7 +437,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. dactyloide</t>
@@ -433,7 +446,7 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">s 'IL' × </t>
@@ -443,7 +456,7 @@
         <i/>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>T. dactyloides</t>
@@ -452,65 +465,10 @@
       <rPr>
         <sz val="7"/>
         <color theme="1"/>
-        <rFont val="Helvetica"/>
+        <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> 'FL'</t>
-    </r>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Proteins quantified</t>
-  </si>
-  <si>
-    <r>
-      <t>3,468
- (4,915</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <t>Shared Winter/Summer</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>before filtering for reproducibility in three out of four batches</t>
     </r>
   </si>
 </sst>
@@ -522,7 +480,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(\ #,##0_);_(\ \(#,##0\);_(\ &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -585,37 +543,36 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="7"/>
       <color rgb="FF000000"/>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color theme="1"/>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color theme="1"/>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="7"/>
       <color rgb="FF000000"/>
-      <name val="Helvetica"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -717,149 +674,149 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1197,7 +1154,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DC014EF-4911-4042-A194-C625793BB42C}">
   <dimension ref="B2:I46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" customWidth="1"/>
@@ -1207,32 +1164,32 @@
     <col min="9" max="9" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="24" customHeight="1">
-      <c r="B2" s="41" t="s">
+    <row r="2" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41" t="s">
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="41" t="s">
+      <c r="I2" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="24" customHeight="1">
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="46"/>
+    <row r="3" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="15"/>
       <c r="E3" s="6" t="s">
         <v>47</v>
       </c>
@@ -1242,17 +1199,17 @@
       <c r="G3" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-    </row>
-    <row r="4" spans="2:9" ht="24" customHeight="1">
-      <c r="B4" s="29" t="s">
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+    </row>
+    <row r="4" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
         <v>51</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="33">
+      <c r="D4" s="21">
         <v>2022</v>
       </c>
       <c r="E4" s="3">
@@ -1261,56 +1218,56 @@
       <c r="F4" s="3">
         <v>3722</v>
       </c>
-      <c r="G4" s="37">
+      <c r="G4" s="20">
         <v>3733</v>
       </c>
-      <c r="H4" s="35">
+      <c r="H4" s="18">
         <v>109</v>
       </c>
-      <c r="I4" s="35">
+      <c r="I4" s="18">
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="24" customHeight="1">
-      <c r="B5" s="29"/>
+    <row r="5" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="27"/>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="33"/>
+      <c r="D5" s="21"/>
       <c r="E5" s="3">
         <v>3734</v>
       </c>
       <c r="F5" s="3">
         <v>3732</v>
       </c>
-      <c r="G5" s="37"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="35"/>
-    </row>
-    <row r="6" spans="2:9" ht="24" customHeight="1">
-      <c r="B6" s="30"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+    </row>
+    <row r="6" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="28"/>
       <c r="C6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="34"/>
+      <c r="D6" s="25"/>
       <c r="E6" s="7">
         <v>3734</v>
       </c>
       <c r="F6" s="7">
         <v>3734</v>
       </c>
-      <c r="G6" s="38"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-    </row>
-    <row r="7" spans="2:9" ht="24" customHeight="1">
-      <c r="B7" s="31" t="s">
+      <c r="G6" s="29"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+    </row>
+    <row r="7" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="23" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="21">
         <v>2022</v>
       </c>
       <c r="E7" s="4">
@@ -1319,56 +1276,56 @@
       <c r="F7" s="4">
         <v>3720</v>
       </c>
-      <c r="G7" s="37">
+      <c r="G7" s="20">
         <v>2273</v>
       </c>
-      <c r="H7" s="35">
+      <c r="H7" s="18">
         <v>58</v>
       </c>
-      <c r="I7" s="35">
+      <c r="I7" s="18">
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="24" customHeight="1">
-      <c r="B8" s="31"/>
+    <row r="8" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="23"/>
       <c r="C8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="33"/>
+      <c r="D8" s="21"/>
       <c r="E8" s="4">
         <v>3691</v>
       </c>
       <c r="F8" s="4">
         <v>3707</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-    </row>
-    <row r="9" spans="2:9" ht="24" customHeight="1">
-      <c r="B9" s="32"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+    </row>
+    <row r="9" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="24"/>
       <c r="C9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="34"/>
+      <c r="D9" s="25"/>
       <c r="E9" s="7">
         <v>3690</v>
       </c>
       <c r="F9" s="7">
         <v>3686</v>
       </c>
-      <c r="G9" s="38"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-    </row>
-    <row r="10" spans="2:9" ht="24" customHeight="1">
-      <c r="B10" s="31" t="s">
+      <c r="G9" s="29"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+    </row>
+    <row r="10" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="23" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="21">
         <v>2022</v>
       </c>
       <c r="E10" s="4">
@@ -1377,56 +1334,56 @@
       <c r="F10" s="4">
         <v>4071</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="20">
         <v>4068</v>
       </c>
-      <c r="H10" s="35">
+      <c r="H10" s="18">
         <v>174</v>
       </c>
-      <c r="I10" s="35">
+      <c r="I10" s="18">
         <v>218</v>
       </c>
     </row>
-    <row r="11" spans="2:9" ht="24" customHeight="1">
-      <c r="B11" s="31"/>
+    <row r="11" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="23"/>
       <c r="C11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="33"/>
+      <c r="D11" s="21"/>
       <c r="E11" s="4">
         <v>4071</v>
       </c>
       <c r="F11" s="4">
         <v>4070</v>
       </c>
-      <c r="G11" s="37"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-    </row>
-    <row r="12" spans="2:9" ht="24" customHeight="1">
-      <c r="B12" s="32"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+    </row>
+    <row r="12" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="24"/>
       <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="34"/>
+      <c r="D12" s="25"/>
       <c r="E12" s="7">
         <v>4071</v>
       </c>
       <c r="F12" s="7">
         <v>4069</v>
       </c>
-      <c r="G12" s="38"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-    </row>
-    <row r="13" spans="2:9" ht="24" customHeight="1">
-      <c r="B13" s="31" t="s">
+      <c r="G12" s="29"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+    </row>
+    <row r="13" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="23" t="s">
         <v>62</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="21">
         <v>2022</v>
       </c>
       <c r="E13" s="4">
@@ -1435,40 +1392,40 @@
       <c r="F13" s="4">
         <v>2369</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="20">
         <v>2464</v>
       </c>
-      <c r="H13" s="35">
+      <c r="H13" s="18">
         <v>66</v>
       </c>
-      <c r="I13" s="35">
+      <c r="I13" s="18">
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="24" customHeight="1">
-      <c r="B14" s="32"/>
+    <row r="14" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="24"/>
       <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="34"/>
+      <c r="D14" s="25"/>
       <c r="E14" s="7">
         <v>2499</v>
       </c>
       <c r="F14" s="7">
         <v>2556</v>
       </c>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-    </row>
-    <row r="15" spans="2:9" ht="24" customHeight="1">
-      <c r="B15" s="31" t="s">
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+    </row>
+    <row r="15" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="23" t="s">
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="21">
         <v>2022</v>
       </c>
       <c r="E15" s="4">
@@ -1477,392 +1434,392 @@
       <c r="F15" s="4">
         <v>3608</v>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="20">
         <v>3054</v>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="18">
         <v>100</v>
       </c>
-      <c r="I15" s="35">
+      <c r="I15" s="18">
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="2:9" ht="24" customHeight="1">
-      <c r="B16" s="31"/>
+    <row r="16" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="23"/>
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="33"/>
+      <c r="D16" s="21"/>
       <c r="E16" s="4">
         <v>3607</v>
       </c>
       <c r="F16" s="4">
         <v>3609</v>
       </c>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-    </row>
-    <row r="17" spans="2:9" ht="24" customHeight="1">
-      <c r="B17" s="31"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+    </row>
+    <row r="17" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="23"/>
       <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="33"/>
+      <c r="D17" s="21"/>
       <c r="E17" s="4">
         <v>3607</v>
       </c>
       <c r="F17" s="4">
         <v>3599</v>
       </c>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-    </row>
-    <row r="18" spans="2:9" ht="24" customHeight="1">
-      <c r="B18" s="31"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+    </row>
+    <row r="18" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="23"/>
       <c r="C18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="33"/>
+      <c r="D18" s="21"/>
       <c r="E18" s="4">
         <v>3608</v>
       </c>
       <c r="F18" s="4">
         <v>3604</v>
       </c>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-    </row>
-    <row r="19" spans="2:9" ht="24" customHeight="1">
-      <c r="B19" s="31"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+    </row>
+    <row r="19" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="23"/>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="33"/>
+      <c r="D19" s="21"/>
       <c r="E19" s="4">
         <v>3608</v>
       </c>
       <c r="F19" s="4">
         <v>3597</v>
       </c>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-    </row>
-    <row r="20" spans="2:9" ht="24" customHeight="1">
-      <c r="B20" s="31"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+    </row>
+    <row r="20" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="23"/>
       <c r="C20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="33"/>
+      <c r="D20" s="21"/>
       <c r="E20" s="4">
         <v>3609</v>
       </c>
       <c r="F20" s="4">
         <v>3598</v>
       </c>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-    </row>
-    <row r="21" spans="2:9" ht="24" customHeight="1">
-      <c r="B21" s="31"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+    </row>
+    <row r="21" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="23"/>
       <c r="C21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="33"/>
+      <c r="D21" s="21"/>
       <c r="E21" s="4">
         <v>3159</v>
       </c>
       <c r="F21" s="4">
         <v>3161</v>
       </c>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-    </row>
-    <row r="22" spans="2:9" ht="24" customHeight="1">
-      <c r="B22" s="31"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+    </row>
+    <row r="22" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="23"/>
       <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="33"/>
+      <c r="D22" s="21"/>
       <c r="E22" s="4">
         <v>3160</v>
       </c>
       <c r="F22" s="4">
         <v>3161</v>
       </c>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-    </row>
-    <row r="23" spans="2:9" ht="24" customHeight="1">
-      <c r="B23" s="31"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+    </row>
+    <row r="23" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="23"/>
       <c r="C23" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="33"/>
+      <c r="D23" s="21"/>
       <c r="E23" s="4">
         <v>3161</v>
       </c>
       <c r="F23" s="4">
         <v>3161</v>
       </c>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-    </row>
-    <row r="24" spans="2:9" ht="24" customHeight="1">
-      <c r="B24" s="31"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+    </row>
+    <row r="24" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="23"/>
       <c r="C24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="33"/>
+      <c r="D24" s="21"/>
       <c r="E24" s="4">
         <v>3800</v>
       </c>
       <c r="F24" s="4">
         <v>3787</v>
       </c>
-      <c r="G24" s="35"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-    </row>
-    <row r="25" spans="2:9" ht="24" customHeight="1">
-      <c r="B25" s="31"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+    </row>
+    <row r="25" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="23"/>
       <c r="C25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="33"/>
+      <c r="D25" s="21"/>
       <c r="E25" s="4">
         <v>3799</v>
       </c>
       <c r="F25" s="4">
         <v>3607</v>
       </c>
-      <c r="G25" s="35"/>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-    </row>
-    <row r="26" spans="2:9" ht="24" customHeight="1">
-      <c r="B26" s="31"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+    </row>
+    <row r="26" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="23"/>
       <c r="C26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="33"/>
+      <c r="D26" s="21"/>
       <c r="E26" s="4">
         <v>3798</v>
       </c>
       <c r="F26" s="4">
         <v>3769</v>
       </c>
-      <c r="G26" s="35"/>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-    </row>
-    <row r="27" spans="2:9" ht="24" customHeight="1">
-      <c r="B27" s="31"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+    </row>
+    <row r="27" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="23"/>
       <c r="C27" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="33"/>
+      <c r="D27" s="21"/>
       <c r="E27" s="4">
         <v>3799</v>
       </c>
       <c r="F27" s="4">
         <v>3790</v>
       </c>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-    </row>
-    <row r="28" spans="2:9" ht="24" customHeight="1">
-      <c r="B28" s="31"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+    </row>
+    <row r="28" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="23"/>
       <c r="C28" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="33"/>
+      <c r="D28" s="21"/>
       <c r="E28" s="4">
         <v>3799</v>
       </c>
       <c r="F28" s="4">
         <v>3770</v>
       </c>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="35"/>
-    </row>
-    <row r="29" spans="2:9" ht="24" customHeight="1">
-      <c r="B29" s="31"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+    </row>
+    <row r="29" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="23"/>
       <c r="C29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="33"/>
+      <c r="D29" s="21"/>
       <c r="E29" s="4">
         <v>3798</v>
       </c>
       <c r="F29" s="4">
         <v>3797</v>
       </c>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-    </row>
-    <row r="30" spans="2:9" ht="24" customHeight="1">
-      <c r="B30" s="31"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="18"/>
+    </row>
+    <row r="30" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="23"/>
       <c r="C30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="33"/>
+      <c r="D30" s="21"/>
       <c r="E30" s="4">
         <v>3474</v>
       </c>
       <c r="F30" s="4">
         <v>3477</v>
       </c>
-      <c r="G30" s="35"/>
-      <c r="H30" s="35"/>
-      <c r="I30" s="35"/>
-    </row>
-    <row r="31" spans="2:9" ht="24" customHeight="1">
-      <c r="B31" s="31"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+    </row>
+    <row r="31" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="23"/>
       <c r="C31" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D31" s="33"/>
+      <c r="D31" s="21"/>
       <c r="E31" s="4">
         <v>3473</v>
       </c>
       <c r="F31" s="4">
         <v>3474</v>
       </c>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-    </row>
-    <row r="32" spans="2:9" ht="24" customHeight="1">
-      <c r="B32" s="31"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+    </row>
+    <row r="32" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="23"/>
       <c r="C32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="33"/>
+      <c r="D32" s="21"/>
       <c r="E32" s="4">
         <v>3474</v>
       </c>
       <c r="F32" s="4">
         <v>3478</v>
       </c>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-    </row>
-    <row r="33" spans="2:9" ht="24" customHeight="1">
-      <c r="B33" s="31"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+    </row>
+    <row r="33" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="23"/>
       <c r="C33" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="33"/>
+      <c r="D33" s="21"/>
       <c r="E33" s="4">
         <v>3475</v>
       </c>
       <c r="F33" s="4">
         <v>3478</v>
       </c>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-    </row>
-    <row r="34" spans="2:9" ht="24" customHeight="1">
-      <c r="B34" s="31"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+    </row>
+    <row r="34" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="23"/>
       <c r="C34" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="33"/>
+      <c r="D34" s="21"/>
       <c r="E34" s="4">
         <v>3477</v>
       </c>
       <c r="F34" s="4">
         <v>3478</v>
       </c>
-      <c r="G34" s="35"/>
-      <c r="H34" s="35"/>
-      <c r="I34" s="35"/>
-    </row>
-    <row r="35" spans="2:9" ht="24" customHeight="1">
-      <c r="B35" s="31"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+    </row>
+    <row r="35" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="23"/>
       <c r="C35" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="33"/>
+      <c r="D35" s="21"/>
       <c r="E35" s="4">
         <v>3476</v>
       </c>
       <c r="F35" s="4">
         <v>3473</v>
       </c>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="35"/>
-    </row>
-    <row r="36" spans="2:9" ht="24" customHeight="1">
-      <c r="B36" s="31"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+    </row>
+    <row r="36" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="23"/>
       <c r="C36" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D36" s="33"/>
+      <c r="D36" s="21"/>
       <c r="E36" s="4">
         <v>3161</v>
       </c>
       <c r="F36" s="4">
         <v>3123</v>
       </c>
-      <c r="G36" s="35"/>
-      <c r="H36" s="35"/>
-      <c r="I36" s="35"/>
-    </row>
-    <row r="37" spans="2:9" ht="24" customHeight="1">
-      <c r="B37" s="31"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+    </row>
+    <row r="37" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="23"/>
       <c r="C37" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="33"/>
+      <c r="D37" s="21"/>
       <c r="E37" s="4">
         <v>3159</v>
       </c>
       <c r="F37" s="4">
         <v>3158</v>
       </c>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-    </row>
-    <row r="38" spans="2:9" ht="24" customHeight="1">
-      <c r="B38" s="32"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+    </row>
+    <row r="38" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="24"/>
       <c r="C38" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="34"/>
+      <c r="D38" s="25"/>
       <c r="E38" s="7">
         <v>3157</v>
       </c>
       <c r="F38" s="7">
         <v>3157</v>
       </c>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-    </row>
-    <row r="39" spans="2:9" ht="24" customHeight="1">
-      <c r="B39" s="39" t="s">
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+    </row>
+    <row r="39" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="16" t="s">
         <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D39" s="33">
+      <c r="D39" s="21">
         <v>2019</v>
       </c>
       <c r="E39" s="4">
@@ -1871,135 +1828,145 @@
       <c r="F39" s="4">
         <v>4451</v>
       </c>
-      <c r="G39" s="37">
+      <c r="G39" s="20">
         <v>4451</v>
       </c>
-      <c r="H39" s="35">
+      <c r="H39" s="18">
         <v>123</v>
       </c>
-      <c r="I39" s="35">
+      <c r="I39" s="18">
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="2:9" ht="24" customHeight="1">
-      <c r="B40" s="39"/>
+    <row r="40" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="16"/>
       <c r="C40" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D40" s="33"/>
+      <c r="D40" s="21"/>
       <c r="E40" s="4">
         <v>4451</v>
       </c>
       <c r="F40" s="4">
         <v>4451</v>
       </c>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="35"/>
-    </row>
-    <row r="41" spans="2:9" ht="24" customHeight="1">
-      <c r="B41" s="39"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+    </row>
+    <row r="41" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="16"/>
       <c r="C41" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D41" s="33"/>
+      <c r="D41" s="21"/>
       <c r="E41" s="4">
         <v>4451</v>
       </c>
       <c r="F41" s="4">
         <v>4451</v>
       </c>
-      <c r="G41" s="35"/>
-      <c r="H41" s="35"/>
-      <c r="I41" s="35"/>
-    </row>
-    <row r="42" spans="2:9" ht="24" customHeight="1">
-      <c r="B42" s="39"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="18"/>
+    </row>
+    <row r="42" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="16"/>
       <c r="C42" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D42" s="33"/>
+      <c r="D42" s="21"/>
       <c r="E42" s="4">
         <v>4451</v>
       </c>
       <c r="F42" s="4">
         <v>4451</v>
       </c>
-      <c r="G42" s="35"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="35"/>
-    </row>
-    <row r="43" spans="2:9" ht="24" customHeight="1">
-      <c r="B43" s="39"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="18"/>
+    </row>
+    <row r="43" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="16"/>
       <c r="C43" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D43" s="33"/>
+      <c r="D43" s="21"/>
       <c r="E43" s="4">
         <v>4451</v>
       </c>
       <c r="F43" s="4">
         <v>4451</v>
       </c>
-      <c r="G43" s="35"/>
-      <c r="H43" s="35"/>
-      <c r="I43" s="35"/>
-    </row>
-    <row r="44" spans="2:9" ht="24" customHeight="1">
-      <c r="B44" s="39"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="18"/>
+    </row>
+    <row r="44" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="16"/>
       <c r="C44" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D44" s="33"/>
+      <c r="D44" s="21"/>
       <c r="E44" s="4">
         <v>4451</v>
       </c>
       <c r="F44" s="4">
         <v>4451</v>
       </c>
-      <c r="G44" s="35"/>
-      <c r="H44" s="35"/>
-      <c r="I44" s="35"/>
-    </row>
-    <row r="45" spans="2:9" ht="24" customHeight="1">
-      <c r="B45" s="39"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="18"/>
+    </row>
+    <row r="45" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="16"/>
       <c r="C45" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D45" s="33"/>
+      <c r="D45" s="21"/>
       <c r="E45" s="4">
         <v>4451</v>
       </c>
       <c r="F45" s="4">
         <v>4451</v>
       </c>
-      <c r="G45" s="35"/>
-      <c r="H45" s="35"/>
-      <c r="I45" s="35"/>
-    </row>
-    <row r="46" spans="2:9" ht="24" customHeight="1">
-      <c r="B46" s="40"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+    </row>
+    <row r="46" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="17"/>
       <c r="C46" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D46" s="43"/>
+      <c r="D46" s="22"/>
       <c r="E46" s="5">
         <v>4451</v>
       </c>
       <c r="F46" s="5">
         <v>4451</v>
       </c>
-      <c r="G46" s="42"/>
-      <c r="H46" s="42"/>
-      <c r="I46" s="42"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="19"/>
+      <c r="I46" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="D7:D9"/>
     <mergeCell ref="B39:B46"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="I39:I46"/>
@@ -2016,21 +1983,11 @@
     <mergeCell ref="H15:H38"/>
     <mergeCell ref="G15:G38"/>
     <mergeCell ref="B15:B38"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="H10:H12"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="I4:I6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="C2:C3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2044,7 +2001,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2055,278 +2012,283 @@
     <col min="7" max="8" width="6.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19" customHeight="1"/>
-    <row r="2" spans="1:8" ht="16" customHeight="1">
-      <c r="A2" s="52" t="s">
+    <row r="1" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="D2" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="32"/>
+      <c r="G2" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="33"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+    </row>
+    <row r="4" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="39">
+        <v>2019</v>
+      </c>
+      <c r="D4" s="39">
+        <v>8</v>
+      </c>
+      <c r="E4" s="40">
+        <v>4451</v>
+      </c>
+      <c r="F4" s="40">
+        <v>4451</v>
+      </c>
+      <c r="G4" s="39">
+        <v>123</v>
+      </c>
+      <c r="H4" s="39">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="41"/>
+      <c r="B5" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+    </row>
+    <row r="6" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="41"/>
+      <c r="B6" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="51"/>
-      <c r="G2" s="52" t="s">
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+    </row>
+    <row r="7" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="43">
+        <v>2022</v>
+      </c>
+      <c r="D7" s="43">
+        <v>24</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="44">
+        <v>3054</v>
+      </c>
+      <c r="G7" s="43">
+        <v>100</v>
+      </c>
+      <c r="H7" s="43">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="41"/>
+      <c r="B8" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+    </row>
+    <row r="9" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="41"/>
+      <c r="B9" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+    </row>
+    <row r="10" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="41"/>
+      <c r="B10" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+    </row>
+    <row r="11" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="41"/>
+      <c r="B11" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="49">
+        <v>2022</v>
+      </c>
+      <c r="D12" s="50">
         <v>3</v>
       </c>
-      <c r="H2" s="52" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="23" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F3" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-    </row>
-    <row r="4" spans="1:8" ht="16" customHeight="1">
-      <c r="A4" s="54" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="55">
-        <v>2019</v>
-      </c>
-      <c r="D4" s="55">
-        <v>8</v>
-      </c>
-      <c r="E4" s="56">
-        <v>4451</v>
-      </c>
-      <c r="F4" s="56">
-        <v>4451</v>
-      </c>
-      <c r="G4" s="55">
-        <v>123</v>
-      </c>
-      <c r="H4" s="55">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="16" customHeight="1">
-      <c r="A5" s="48"/>
-      <c r="B5" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
-    </row>
-    <row r="6" spans="1:8" ht="16" customHeight="1">
-      <c r="A6" s="48"/>
-      <c r="B6" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-    </row>
-    <row r="7" spans="1:8" ht="16" customHeight="1">
-      <c r="A7" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="47">
+      <c r="E12" s="51">
+        <v>3734</v>
+      </c>
+      <c r="F12" s="51">
+        <v>3733</v>
+      </c>
+      <c r="G12" s="49">
+        <v>109</v>
+      </c>
+      <c r="H12" s="49">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="42"/>
+      <c r="C13" s="49">
         <v>2022</v>
       </c>
-      <c r="D7" s="47">
-        <v>24</v>
-      </c>
-      <c r="E7" s="50" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" s="49">
-        <v>3054</v>
-      </c>
-      <c r="G7" s="47">
-        <v>100</v>
-      </c>
-      <c r="H7" s="47">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="16" customHeight="1">
-      <c r="A8" s="48"/>
-      <c r="B8" s="14" t="s">
+      <c r="D13" s="50">
+        <v>3</v>
+      </c>
+      <c r="E13" s="51">
+        <v>2372</v>
+      </c>
+      <c r="F13" s="53">
+        <v>2273</v>
+      </c>
+      <c r="G13" s="49">
+        <v>58</v>
+      </c>
+      <c r="H13" s="49">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="52" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="49">
+        <v>2022</v>
+      </c>
+      <c r="D14" s="50">
+        <v>3</v>
+      </c>
+      <c r="E14" s="51">
+        <v>4071</v>
+      </c>
+      <c r="F14" s="53">
+        <v>4068</v>
+      </c>
+      <c r="G14" s="49">
+        <v>174</v>
+      </c>
+      <c r="H14" s="49">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="54" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="55" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="56">
+        <v>2022</v>
+      </c>
+      <c r="D15" s="57">
+        <v>2</v>
+      </c>
+      <c r="E15" s="58">
+        <v>2641</v>
+      </c>
+      <c r="F15" s="58">
+        <v>2464</v>
+      </c>
+      <c r="G15" s="56">
         <v>66</v>
       </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-    </row>
-    <row r="9" spans="1:8" ht="16" customHeight="1">
-      <c r="A9" s="48"/>
-      <c r="B9" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="47"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="47"/>
-    </row>
-    <row r="10" spans="1:8" ht="16" customHeight="1">
-      <c r="A10" s="48"/>
-      <c r="B10" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-    </row>
-    <row r="11" spans="1:8" ht="16" customHeight="1">
-      <c r="A11" s="48"/>
-      <c r="B11" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="19">
-        <v>2022</v>
-      </c>
-      <c r="D12" s="15">
-        <v>3</v>
-      </c>
-      <c r="E12" s="20">
-        <v>3734</v>
-      </c>
-      <c r="F12" s="20">
-        <v>3733</v>
-      </c>
-      <c r="G12" s="19">
-        <v>109</v>
-      </c>
-      <c r="H12" s="19">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="19">
-        <v>2022</v>
-      </c>
-      <c r="D13" s="15">
-        <v>3</v>
-      </c>
-      <c r="E13" s="20">
-        <v>2372</v>
-      </c>
-      <c r="F13" s="16">
-        <v>2273</v>
-      </c>
-      <c r="G13" s="19">
-        <v>58</v>
-      </c>
-      <c r="H13" s="19">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="21" t="s">
+      <c r="H15" s="56">
         <v>56</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="19">
-        <v>2022</v>
-      </c>
-      <c r="D14" s="15">
-        <v>3</v>
-      </c>
-      <c r="E14" s="20">
-        <v>4071</v>
-      </c>
-      <c r="F14" s="16">
-        <v>4068</v>
-      </c>
-      <c r="G14" s="19">
-        <v>174</v>
-      </c>
-      <c r="H14" s="19">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="16" customHeight="1">
-      <c r="A15" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="24">
-        <v>2022</v>
-      </c>
-      <c r="D15" s="25">
-        <v>2</v>
-      </c>
-      <c r="E15" s="26">
-        <v>2641</v>
-      </c>
-      <c r="F15" s="26">
-        <v>2464</v>
-      </c>
-      <c r="G15" s="24">
-        <v>66</v>
-      </c>
-      <c r="H15" s="24">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="28" t="s">
-        <v>72</v>
-      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="G7:G11"/>
+    <mergeCell ref="H7:H11"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="D7:D11"/>
+    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="E7:E11"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="H2:H3"/>
@@ -2341,13 +2303,6 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="H4:H6"/>
     <mergeCell ref="E4:E6"/>
-    <mergeCell ref="G7:G11"/>
-    <mergeCell ref="H7:H11"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D11"/>
-    <mergeCell ref="F7:F11"/>
-    <mergeCell ref="E7:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="99" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2357,17 +2312,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25417206-27C8-B34E-A1F3-B483FF5469CF}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="10"/>
       <c r="B1" s="10"/>
     </row>
-    <row r="15" spans="1:2" ht="17" thickBot="1">
+    <row r="15" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
     </row>

</xml_diff>

<commit_message>
Update manuscript, README, figures, and supplemental tables for submission
</commit_message>
<xml_diff>
--- a/tables/Table1_Species_protemics_Summary_table_rev7.xlsx
+++ b/tables/Table1_Species_protemics_Summary_table_rev7.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/211a55de1c355a5b/Projects/BucklerLab/PACMAD-Rhizome-Proteomics/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{3D108CAD-EFD0-5441-84A0-8060CACB3BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F976B7E-DC08-7F4A-8012-5E78D3B36AE7}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="8_{3D108CAD-EFD0-5441-84A0-8060CACB3BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20DA0FB9-1BD3-244F-8A98-AF7B39A15A8F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" activeTab="1" xr2:uid="{E31260A5-6BF7-4247-931C-1F444D52B9F8}"/>
+    <workbookView xWindow="11820" yWindow="-24740" windowWidth="30280" windowHeight="24740" activeTab="1" xr2:uid="{E31260A5-6BF7-4247-931C-1F444D52B9F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,9 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Main table'!$A$2:$H$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Main table'!$A$2:$J$21</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="89">
   <si>
     <t>Species</t>
   </si>
@@ -271,13 +271,142 @@
     <t>Proteins quantified</t>
   </si>
   <si>
-    <t>Shared Winter/Summer</t>
-  </si>
-  <si>
     <t xml:space="preserve">3,468
 </t>
   </si>
   <si>
+    <t>Genotype</t>
+  </si>
+  <si>
+    <t>Entry code</t>
+  </si>
+  <si>
+    <t>Clonal reps</t>
+  </si>
+  <si>
+    <t>Sig up</t>
+  </si>
+  <si>
+    <t>Shared winter/summer</t>
+  </si>
+  <si>
+    <t>C027</t>
+  </si>
+  <si>
+    <t>C043</t>
+  </si>
+  <si>
+    <t>C065</t>
+  </si>
+  <si>
+    <t>C071</t>
+  </si>
+  <si>
+    <t>01-277*B</t>
+  </si>
+  <si>
+    <t>01-266*A</t>
+  </si>
+  <si>
+    <t>88-363*A</t>
+  </si>
+  <si>
+    <t>22-095*A</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. dactyloides</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 'KS_C9_9' × </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. floridanium</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. dactyloides</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 'KS_B6_1' × </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. floridanium</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. dactyloides</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 'KS_C9_10' × </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>T. floridanium</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t>T. dactyloides '</t>
     </r>
@@ -288,7 +417,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>KS'</t>
+      <t>IA_Pete_2'</t>
     </r>
     <r>
       <rPr>
@@ -319,7 +448,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>'IA'</t>
+      <t>'IA_Pete_1'</t>
     </r>
     <r>
       <rPr>
@@ -361,6 +490,9 @@
     </r>
   </si>
   <si>
+    <t>T. dactyloides 'IA_Pete_2' × T. floridanium</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <i/>
@@ -378,7 +510,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> 'MO' × </t>
+      <t xml:space="preserve"> 'KS_C7_3' × </t>
     </r>
     <r>
       <rPr>
@@ -388,6 +520,18 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t>T. floridanium</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>T. dactyloides</t>
     </r>
     <r>
@@ -397,10 +541,8 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> 'TX'</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve"> 'IL_10_1' × </t>
+    </r>
     <r>
       <rPr>
         <i/>
@@ -409,6 +551,77 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t>T. floridanium</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">T. dactyloides </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>'IL_14'</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>×</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> T. dactyloides</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 'FL'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t>T. dactyloides</t>
     </r>
     <r>
@@ -418,7 +631,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> 'IL' × </t>
+      <t xml:space="preserve"> 'TX_HC_3' × </t>
     </r>
     <r>
       <rPr>
@@ -428,37 +641,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>T. floridanium</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>T. dactyloide</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">s 'IL' × </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t>T. dactyloides</t>
     </r>
     <r>
@@ -468,7 +650,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> 'FL'</t>
+      <t xml:space="preserve"> 'MO_TP'</t>
     </r>
   </si>
 </sst>
@@ -644,7 +826,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -677,9 +859,105 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -689,135 +967,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1165,31 +1354,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12" t="s">
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="42" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="15"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="47"/>
       <c r="E3" s="6" t="s">
         <v>47</v>
       </c>
@@ -1199,17 +1388,17 @@
       <c r="G3" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
     </row>
     <row r="4" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="30" t="s">
         <v>51</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="34">
         <v>2022</v>
       </c>
       <c r="E4" s="3">
@@ -1218,56 +1407,56 @@
       <c r="F4" s="3">
         <v>3722</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="38">
         <v>3733</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="36">
         <v>109</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="36">
         <v>76</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="27"/>
+      <c r="B5" s="30"/>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="21"/>
+      <c r="D5" s="34"/>
       <c r="E5" s="3">
         <v>3734</v>
       </c>
       <c r="F5" s="3">
         <v>3732</v>
       </c>
-      <c r="G5" s="20"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
     </row>
     <row r="6" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="28"/>
+      <c r="B6" s="31"/>
       <c r="C6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="25"/>
+      <c r="D6" s="35"/>
       <c r="E6" s="7">
         <v>3734</v>
       </c>
       <c r="F6" s="7">
         <v>3734</v>
       </c>
-      <c r="G6" s="29"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
     </row>
     <row r="7" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="32" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="34">
         <v>2022</v>
       </c>
       <c r="E7" s="4">
@@ -1276,56 +1465,56 @@
       <c r="F7" s="4">
         <v>3720</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="38">
         <v>2273</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="36">
         <v>58</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="36">
         <v>83</v>
       </c>
     </row>
     <row r="8" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="23"/>
+      <c r="B8" s="32"/>
       <c r="C8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="21"/>
+      <c r="D8" s="34"/>
       <c r="E8" s="4">
         <v>3691</v>
       </c>
       <c r="F8" s="4">
         <v>3707</v>
       </c>
-      <c r="G8" s="20"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
     </row>
     <row r="9" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="24"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="25"/>
+      <c r="D9" s="35"/>
       <c r="E9" s="7">
         <v>3690</v>
       </c>
       <c r="F9" s="7">
         <v>3686</v>
       </c>
-      <c r="G9" s="29"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
     </row>
     <row r="10" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="32" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="34">
         <v>2022</v>
       </c>
       <c r="E10" s="4">
@@ -1334,56 +1523,56 @@
       <c r="F10" s="4">
         <v>4071</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="38">
         <v>4068</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="36">
         <v>174</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="36">
         <v>218</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="23"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="21"/>
+      <c r="D11" s="34"/>
       <c r="E11" s="4">
         <v>4071</v>
       </c>
       <c r="F11" s="4">
         <v>4070</v>
       </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
     </row>
     <row r="12" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="24"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="25"/>
+      <c r="D12" s="35"/>
       <c r="E12" s="7">
         <v>4071</v>
       </c>
       <c r="F12" s="7">
         <v>4069</v>
       </c>
-      <c r="G12" s="29"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
     </row>
     <row r="13" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="32" t="s">
         <v>62</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="34">
         <v>2022</v>
       </c>
       <c r="E13" s="4">
@@ -1392,40 +1581,40 @@
       <c r="F13" s="4">
         <v>2369</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="38">
         <v>2464</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="36">
         <v>66</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="36">
         <v>56</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="24"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="25"/>
+      <c r="D14" s="35"/>
       <c r="E14" s="7">
         <v>2499</v>
       </c>
       <c r="F14" s="7">
         <v>2556</v>
       </c>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
     </row>
     <row r="15" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="32" t="s">
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="34">
         <v>2022</v>
       </c>
       <c r="E15" s="4">
@@ -1434,392 +1623,392 @@
       <c r="F15" s="4">
         <v>3608</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="38">
         <v>3054</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="36">
         <v>100</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="36">
         <v>141</v>
       </c>
     </row>
     <row r="16" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="23"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="21"/>
+      <c r="D16" s="34"/>
       <c r="E16" s="4">
         <v>3607</v>
       </c>
       <c r="F16" s="4">
         <v>3609</v>
       </c>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="36"/>
     </row>
     <row r="17" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="23"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="21"/>
+      <c r="D17" s="34"/>
       <c r="E17" s="4">
         <v>3607</v>
       </c>
       <c r="F17" s="4">
         <v>3599</v>
       </c>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="36"/>
     </row>
     <row r="18" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="23"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="21"/>
+      <c r="D18" s="34"/>
       <c r="E18" s="4">
         <v>3608</v>
       </c>
       <c r="F18" s="4">
         <v>3604</v>
       </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="36"/>
     </row>
     <row r="19" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="23"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="21"/>
+      <c r="D19" s="34"/>
       <c r="E19" s="4">
         <v>3608</v>
       </c>
       <c r="F19" s="4">
         <v>3597</v>
       </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
     </row>
     <row r="20" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="23"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="21"/>
+      <c r="D20" s="34"/>
       <c r="E20" s="4">
         <v>3609</v>
       </c>
       <c r="F20" s="4">
         <v>3598</v>
       </c>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
     </row>
     <row r="21" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="23"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="21"/>
+      <c r="D21" s="34"/>
       <c r="E21" s="4">
         <v>3159</v>
       </c>
       <c r="F21" s="4">
         <v>3161</v>
       </c>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
     </row>
     <row r="22" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="23"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="21"/>
+      <c r="D22" s="34"/>
       <c r="E22" s="4">
         <v>3160</v>
       </c>
       <c r="F22" s="4">
         <v>3161</v>
       </c>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
     </row>
     <row r="23" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="23"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="21"/>
+      <c r="D23" s="34"/>
       <c r="E23" s="4">
         <v>3161</v>
       </c>
       <c r="F23" s="4">
         <v>3161</v>
       </c>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
     </row>
     <row r="24" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="23"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="21"/>
+      <c r="D24" s="34"/>
       <c r="E24" s="4">
         <v>3800</v>
       </c>
       <c r="F24" s="4">
         <v>3787</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
     </row>
     <row r="25" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="23"/>
+      <c r="B25" s="32"/>
       <c r="C25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="21"/>
+      <c r="D25" s="34"/>
       <c r="E25" s="4">
         <v>3799</v>
       </c>
       <c r="F25" s="4">
         <v>3607</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
     </row>
     <row r="26" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="23"/>
+      <c r="B26" s="32"/>
       <c r="C26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="21"/>
+      <c r="D26" s="34"/>
       <c r="E26" s="4">
         <v>3798</v>
       </c>
       <c r="F26" s="4">
         <v>3769</v>
       </c>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
     </row>
     <row r="27" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="23"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="21"/>
+      <c r="D27" s="34"/>
       <c r="E27" s="4">
         <v>3799</v>
       </c>
       <c r="F27" s="4">
         <v>3790</v>
       </c>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
     </row>
     <row r="28" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="23"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="21"/>
+      <c r="D28" s="34"/>
       <c r="E28" s="4">
         <v>3799</v>
       </c>
       <c r="F28" s="4">
         <v>3770</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="36"/>
     </row>
     <row r="29" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="23"/>
+      <c r="B29" s="32"/>
       <c r="C29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="21"/>
+      <c r="D29" s="34"/>
       <c r="E29" s="4">
         <v>3798</v>
       </c>
       <c r="F29" s="4">
         <v>3797</v>
       </c>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="36"/>
     </row>
     <row r="30" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="23"/>
+      <c r="B30" s="32"/>
       <c r="C30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="21"/>
+      <c r="D30" s="34"/>
       <c r="E30" s="4">
         <v>3474</v>
       </c>
       <c r="F30" s="4">
         <v>3477</v>
       </c>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="36"/>
     </row>
     <row r="31" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="23"/>
+      <c r="B31" s="32"/>
       <c r="C31" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D31" s="21"/>
+      <c r="D31" s="34"/>
       <c r="E31" s="4">
         <v>3473</v>
       </c>
       <c r="F31" s="4">
         <v>3474</v>
       </c>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="36"/>
     </row>
     <row r="32" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="23"/>
+      <c r="B32" s="32"/>
       <c r="C32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="21"/>
+      <c r="D32" s="34"/>
       <c r="E32" s="4">
         <v>3474</v>
       </c>
       <c r="F32" s="4">
         <v>3478</v>
       </c>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="36"/>
     </row>
     <row r="33" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="23"/>
+      <c r="B33" s="32"/>
       <c r="C33" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="21"/>
+      <c r="D33" s="34"/>
       <c r="E33" s="4">
         <v>3475</v>
       </c>
       <c r="F33" s="4">
         <v>3478</v>
       </c>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="36"/>
     </row>
     <row r="34" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="23"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="21"/>
+      <c r="D34" s="34"/>
       <c r="E34" s="4">
         <v>3477</v>
       </c>
       <c r="F34" s="4">
         <v>3478</v>
       </c>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="18"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="36"/>
     </row>
     <row r="35" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="23"/>
+      <c r="B35" s="32"/>
       <c r="C35" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="21"/>
+      <c r="D35" s="34"/>
       <c r="E35" s="4">
         <v>3476</v>
       </c>
       <c r="F35" s="4">
         <v>3473</v>
       </c>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
+      <c r="I35" s="36"/>
     </row>
     <row r="36" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="23"/>
+      <c r="B36" s="32"/>
       <c r="C36" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D36" s="21"/>
+      <c r="D36" s="34"/>
       <c r="E36" s="4">
         <v>3161</v>
       </c>
       <c r="F36" s="4">
         <v>3123</v>
       </c>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="36"/>
     </row>
     <row r="37" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="23"/>
+      <c r="B37" s="32"/>
       <c r="C37" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="21"/>
+      <c r="D37" s="34"/>
       <c r="E37" s="4">
         <v>3159</v>
       </c>
       <c r="F37" s="4">
         <v>3158</v>
       </c>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="18"/>
+      <c r="G37" s="36"/>
+      <c r="H37" s="36"/>
+      <c r="I37" s="36"/>
     </row>
     <row r="38" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="24"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="25"/>
+      <c r="D38" s="35"/>
       <c r="E38" s="7">
         <v>3157</v>
       </c>
       <c r="F38" s="7">
         <v>3157</v>
       </c>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+      <c r="I38" s="37"/>
     </row>
     <row r="39" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="40" t="s">
         <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="34">
         <v>2019</v>
       </c>
       <c r="E39" s="4">
@@ -1828,145 +2017,135 @@
       <c r="F39" s="4">
         <v>4451</v>
       </c>
-      <c r="G39" s="20">
+      <c r="G39" s="38">
         <v>4451</v>
       </c>
-      <c r="H39" s="18">
+      <c r="H39" s="36">
         <v>123</v>
       </c>
-      <c r="I39" s="18">
+      <c r="I39" s="36">
         <v>175</v>
       </c>
     </row>
     <row r="40" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="16"/>
+      <c r="B40" s="40"/>
       <c r="C40" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D40" s="21"/>
+      <c r="D40" s="34"/>
       <c r="E40" s="4">
         <v>4451</v>
       </c>
       <c r="F40" s="4">
         <v>4451</v>
       </c>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
-      <c r="I40" s="18"/>
+      <c r="G40" s="36"/>
+      <c r="H40" s="36"/>
+      <c r="I40" s="36"/>
     </row>
     <row r="41" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="16"/>
+      <c r="B41" s="40"/>
       <c r="C41" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D41" s="21"/>
+      <c r="D41" s="34"/>
       <c r="E41" s="4">
         <v>4451</v>
       </c>
       <c r="F41" s="4">
         <v>4451</v>
       </c>
-      <c r="G41" s="18"/>
-      <c r="H41" s="18"/>
-      <c r="I41" s="18"/>
+      <c r="G41" s="36"/>
+      <c r="H41" s="36"/>
+      <c r="I41" s="36"/>
     </row>
     <row r="42" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="16"/>
+      <c r="B42" s="40"/>
       <c r="C42" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D42" s="21"/>
+      <c r="D42" s="34"/>
       <c r="E42" s="4">
         <v>4451</v>
       </c>
       <c r="F42" s="4">
         <v>4451</v>
       </c>
-      <c r="G42" s="18"/>
-      <c r="H42" s="18"/>
-      <c r="I42" s="18"/>
+      <c r="G42" s="36"/>
+      <c r="H42" s="36"/>
+      <c r="I42" s="36"/>
     </row>
     <row r="43" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="16"/>
+      <c r="B43" s="40"/>
       <c r="C43" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D43" s="21"/>
+      <c r="D43" s="34"/>
       <c r="E43" s="4">
         <v>4451</v>
       </c>
       <c r="F43" s="4">
         <v>4451</v>
       </c>
-      <c r="G43" s="18"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="18"/>
+      <c r="G43" s="36"/>
+      <c r="H43" s="36"/>
+      <c r="I43" s="36"/>
     </row>
     <row r="44" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="16"/>
+      <c r="B44" s="40"/>
       <c r="C44" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D44" s="21"/>
+      <c r="D44" s="34"/>
       <c r="E44" s="4">
         <v>4451</v>
       </c>
       <c r="F44" s="4">
         <v>4451</v>
       </c>
-      <c r="G44" s="18"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
     </row>
     <row r="45" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="16"/>
+      <c r="B45" s="40"/>
       <c r="C45" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D45" s="21"/>
+      <c r="D45" s="34"/>
       <c r="E45" s="4">
         <v>4451</v>
       </c>
       <c r="F45" s="4">
         <v>4451</v>
       </c>
-      <c r="G45" s="18"/>
-      <c r="H45" s="18"/>
-      <c r="I45" s="18"/>
+      <c r="G45" s="36"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="36"/>
     </row>
     <row r="46" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="17"/>
+      <c r="B46" s="41"/>
       <c r="C46" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D46" s="22"/>
+      <c r="D46" s="44"/>
       <c r="E46" s="5">
         <v>4451</v>
       </c>
       <c r="F46" s="5">
         <v>4451</v>
       </c>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
+      <c r="G46" s="43"/>
+      <c r="H46" s="43"/>
+      <c r="I46" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="H10:H12"/>
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="I4:I6"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="B39:B46"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="I39:I46"/>
@@ -1983,11 +2162,21 @@
     <mergeCell ref="H15:H38"/>
     <mergeCell ref="G15:G38"/>
     <mergeCell ref="B15:B38"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="G7:G9"/>
+    <mergeCell ref="D7:D9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2000,309 +2189,500 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="5.33203125" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" customWidth="1"/>
-    <col min="5" max="5" width="7.6640625" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" customWidth="1"/>
-    <col min="7" max="8" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="4" width="5.33203125" customWidth="1"/>
+    <col min="5" max="5" width="4.33203125" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" customWidth="1"/>
+    <col min="7" max="7" width="7.6640625" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" customWidth="1"/>
+    <col min="9" max="10" width="6.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="s">
+    <row r="1" spans="1:10" ht="19" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="58" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="58" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="52"/>
+      <c r="I2" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="53" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="54"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+    </row>
+    <row r="4" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="56">
+        <v>2019</v>
+      </c>
+      <c r="E4" s="15">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="30" t="s">
+      <c r="F4" s="56">
+        <v>8</v>
+      </c>
+      <c r="G4" s="57">
+        <v>4451</v>
+      </c>
+      <c r="H4" s="57">
+        <v>4451</v>
+      </c>
+      <c r="I4" s="56">
+        <v>123</v>
+      </c>
+      <c r="J4" s="56">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="49"/>
+      <c r="B5" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="48"/>
+      <c r="E5" s="18">
+        <v>1</v>
+      </c>
+      <c r="F5" s="48"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+    </row>
+    <row r="6" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="49"/>
+      <c r="B6" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="48"/>
+      <c r="E6" s="18">
         <v>3</v>
       </c>
-      <c r="H2" s="30" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="23" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="33"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="35" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3" s="36" t="s">
+      <c r="F6" s="48"/>
+      <c r="G6" s="50"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+    </row>
+    <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="49"/>
+      <c r="B7" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="48"/>
+      <c r="E7" s="18">
+        <v>1</v>
+      </c>
+      <c r="F7" s="48"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+    </row>
+    <row r="8" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="49"/>
+      <c r="B8" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="48"/>
+      <c r="E8" s="18">
+        <v>1</v>
+      </c>
+      <c r="F8" s="48"/>
+      <c r="G8" s="50"/>
+      <c r="H8" s="50"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+    </row>
+    <row r="9" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="49"/>
+      <c r="B9" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="48"/>
+      <c r="E9" s="18">
+        <v>1</v>
+      </c>
+      <c r="F9" s="48"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+    </row>
+    <row r="10" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="48">
+        <v>2022</v>
+      </c>
+      <c r="E10" s="18">
+        <v>3</v>
+      </c>
+      <c r="F10" s="48">
+        <v>24</v>
+      </c>
+      <c r="G10" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-    </row>
-    <row r="4" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" s="39">
-        <v>2019</v>
-      </c>
-      <c r="D4" s="39">
-        <v>8</v>
-      </c>
-      <c r="E4" s="40">
-        <v>4451</v>
-      </c>
-      <c r="F4" s="40">
-        <v>4451</v>
-      </c>
-      <c r="G4" s="39">
-        <v>123</v>
-      </c>
-      <c r="H4" s="39">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="41"/>
-      <c r="B5" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-    </row>
-    <row r="6" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="41"/>
-      <c r="B6" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="43"/>
-    </row>
-    <row r="7" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="B7" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="43">
+      <c r="H10" s="50">
+        <v>3054</v>
+      </c>
+      <c r="I10" s="48">
+        <v>100</v>
+      </c>
+      <c r="J10" s="48">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="49"/>
+      <c r="B11" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="48"/>
+      <c r="E11" s="18">
+        <v>3</v>
+      </c>
+      <c r="F11" s="48"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="50"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
+    </row>
+    <row r="12" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="49"/>
+      <c r="B12" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="48"/>
+      <c r="E12" s="18">
+        <v>3</v>
+      </c>
+      <c r="F12" s="48"/>
+      <c r="G12" s="51"/>
+      <c r="H12" s="50"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="48"/>
+    </row>
+    <row r="13" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="49"/>
+      <c r="B13" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="48"/>
+      <c r="E13" s="18">
+        <v>3</v>
+      </c>
+      <c r="F13" s="48"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="48"/>
+    </row>
+    <row r="14" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="49"/>
+      <c r="B14" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="48"/>
+      <c r="E14" s="18">
+        <v>3</v>
+      </c>
+      <c r="F14" s="48"/>
+      <c r="G14" s="51"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+    </row>
+    <row r="15" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="49"/>
+      <c r="B15" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="48"/>
+      <c r="E15" s="18">
+        <v>3</v>
+      </c>
+      <c r="F15" s="48"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="48"/>
+    </row>
+    <row r="16" spans="1:10" s="61" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="49"/>
+      <c r="B16" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="48"/>
+      <c r="E16" s="18">
+        <v>3</v>
+      </c>
+      <c r="F16" s="48"/>
+      <c r="G16" s="51"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="48"/>
+    </row>
+    <row r="17" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="49"/>
+      <c r="B17" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="48"/>
+      <c r="E17" s="18">
+        <v>3</v>
+      </c>
+      <c r="F17" s="48"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="48"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="22">
         <v>2022</v>
       </c>
-      <c r="D7" s="43">
-        <v>24</v>
-      </c>
-      <c r="E7" s="46" t="s">
+      <c r="E18" s="22">
+        <v>3</v>
+      </c>
+      <c r="F18" s="18">
+        <v>3</v>
+      </c>
+      <c r="G18" s="23">
+        <v>3734</v>
+      </c>
+      <c r="H18" s="23">
+        <v>3733</v>
+      </c>
+      <c r="I18" s="22">
+        <v>109</v>
+      </c>
+      <c r="J18" s="22">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="22">
+        <v>2022</v>
+      </c>
+      <c r="E19" s="22">
+        <v>3</v>
+      </c>
+      <c r="F19" s="18">
+        <v>3</v>
+      </c>
+      <c r="G19" s="23">
+        <v>2372</v>
+      </c>
+      <c r="H19" s="19">
+        <v>2273</v>
+      </c>
+      <c r="I19" s="22">
+        <v>58</v>
+      </c>
+      <c r="J19" s="22">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="22">
+        <v>2022</v>
+      </c>
+      <c r="E20" s="22">
+        <v>3</v>
+      </c>
+      <c r="F20" s="18">
+        <v>3</v>
+      </c>
+      <c r="G20" s="23">
+        <v>4071</v>
+      </c>
+      <c r="H20" s="19">
+        <v>4068</v>
+      </c>
+      <c r="I20" s="22">
+        <v>174</v>
+      </c>
+      <c r="J20" s="22">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="27">
+        <v>2022</v>
+      </c>
+      <c r="E21" s="27">
+        <v>2</v>
+      </c>
+      <c r="F21" s="28">
+        <v>2</v>
+      </c>
+      <c r="G21" s="29">
+        <v>2641</v>
+      </c>
+      <c r="H21" s="29">
+        <v>2464</v>
+      </c>
+      <c r="I21" s="27">
         <v>66</v>
       </c>
-      <c r="F7" s="44">
-        <v>3054</v>
-      </c>
-      <c r="G7" s="43">
-        <v>100</v>
-      </c>
-      <c r="H7" s="43">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="41"/>
-      <c r="B8" s="42" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-    </row>
-    <row r="9" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="41"/>
-      <c r="B9" s="42" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
-    </row>
-    <row r="10" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="41"/>
-      <c r="B10" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-    </row>
-    <row r="11" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="41"/>
-      <c r="B11" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="47" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="49">
-        <v>2022</v>
-      </c>
-      <c r="D12" s="50">
-        <v>3</v>
-      </c>
-      <c r="E12" s="51">
-        <v>3734</v>
-      </c>
-      <c r="F12" s="51">
-        <v>3733</v>
-      </c>
-      <c r="G12" s="49">
-        <v>109</v>
-      </c>
-      <c r="H12" s="49">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="49">
-        <v>2022</v>
-      </c>
-      <c r="D13" s="50">
-        <v>3</v>
-      </c>
-      <c r="E13" s="51">
-        <v>2372</v>
-      </c>
-      <c r="F13" s="53">
-        <v>2273</v>
-      </c>
-      <c r="G13" s="49">
-        <v>58</v>
-      </c>
-      <c r="H13" s="49">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="52" t="s">
+      <c r="J21" s="27">
         <v>56</v>
       </c>
-      <c r="B14" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="49">
-        <v>2022</v>
-      </c>
-      <c r="D14" s="50">
-        <v>3</v>
-      </c>
-      <c r="E14" s="51">
-        <v>4071</v>
-      </c>
-      <c r="F14" s="53">
-        <v>4068</v>
-      </c>
-      <c r="G14" s="49">
-        <v>174</v>
-      </c>
-      <c r="H14" s="49">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="55" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="56">
-        <v>2022</v>
-      </c>
-      <c r="D15" s="57">
-        <v>2</v>
-      </c>
-      <c r="E15" s="58">
-        <v>2641</v>
-      </c>
-      <c r="F15" s="58">
-        <v>2464</v>
-      </c>
-      <c r="G15" s="56">
-        <v>66</v>
-      </c>
-      <c r="H15" s="56">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="G7:G11"/>
-    <mergeCell ref="H7:H11"/>
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="D7:D11"/>
-    <mergeCell ref="F7:F11"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="G4:G6"/>
+  <mergeCells count="23">
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="A4:A9"/>
+    <mergeCell ref="D4:D9"/>
+    <mergeCell ref="F4:F9"/>
+    <mergeCell ref="H4:H9"/>
+    <mergeCell ref="I4:I9"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="J4:J9"/>
+    <mergeCell ref="G4:G9"/>
+    <mergeCell ref="E2:E3"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="I10:I17"/>
+    <mergeCell ref="J10:J17"/>
+    <mergeCell ref="A10:A17"/>
+    <mergeCell ref="D10:D17"/>
+    <mergeCell ref="F10:F17"/>
+    <mergeCell ref="H10:H17"/>
+    <mergeCell ref="G10:G17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="99" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>